<commit_message>
feat(courseware): align Lumina Copilot labs and visual workflow
</commit_message>
<xml_diff>
--- a/activities/lab-01-set-up-and-prompt-safely/Lumina-Living-Lab-01.xlsx
+++ b/activities/lab-01-set-up-and-prompt-safely/Lumina-Living-Lab-01.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Scenario" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Prompt_Log" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Evidence_Register" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Acceptance_Check" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Connected_Workflow" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Scenario" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Prompt_Log" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Evidence_Register" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Acceptance_Check" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Acceptance_Check!$A$1:$D$2</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Evidence_Register!$A$1:$G$5</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Prompt_Log!$A$1:$F$2</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Scenario!$A$1:$H$10</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Acceptance_Check!$A$1:$D$2</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Evidence_Register!$A$1:$G$5</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Prompt_Log!$A$1:$F$2</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Scenario!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +30,70 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="64">
+  <si>
+    <t xml:space="preserve">Field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lumina Living Pte Ltd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SW-2026 Sustainable Workspace Launch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project intake and source register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lumina-Company-Brief.docx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SW-2026-Source-Register.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identify the project objective, four department owners, source authority and missing facts. Compare a vague prompt with a complete Goal–Context–Source–Expectations prompt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Context</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You work for Lumina Living Pte Ltd on SW-2026, the Sustainable Workspace Launch. HR, Marketing, Finance and Operations share one evidence trail. Launch is planned for 1 October 2026; budget SGD 18,000; target 120 qualified enquiries.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lumina-Company-Brief.docx. Use your own reviewed prior-lab files first; scenario/ contains supplied fallback examples.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expectations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Save SW-2026-Source-Register.xlsx. Record source version, verified facts, unresolved questions and reviewer in Lumina-Living-Lab-01.xlsx. Keep projectSW-2026 and action IDsA01–A04 unchanged. Label every output Draft until reviewed; record actual app actions separately.</t>
+  </si>
   <si>
     <t xml:space="preserve">Lab 01: Set Up Microsoft 365 Copilot and Prompt Safely</t>
   </si>
@@ -55,9 +119,6 @@
     <t xml:space="preserve">Microsoft 365 Copilot Chat + Excel</t>
   </si>
   <si>
-    <t xml:space="preserve">Goal</t>
-  </si>
-  <si>
     <t xml:space="preserve">Establish the licensed work surface, distinguish work from web grounding and record safe-use controls.</t>
   </si>
   <si>
@@ -73,9 +134,6 @@
     <t xml:space="preserve">K1 · A1</t>
   </si>
   <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
     <t xml:space="preserve">Learner starter</t>
   </si>
   <si>
@@ -100,7 +158,10 @@
     <t xml:space="preserve">Set Up Microsoft 365 Copilot and Prompt Safely</t>
   </si>
   <si>
-    <t xml:space="preserve">Using the attached workbook and only the information it contains, summarise the three highest-priority readiness gaps for Lumina Living. For each gap, cite the sheet and row evidence, state the risk, propose one control, and label anything you cannot verify.</t>
+    <t xml:space="preserve">Goal: Identify the project objective, four department owners, source authority and missing facts. Compare a vague prompt with a complete Goal–Context–Source–Expectations prompt.
+Context: You work for Lumina Living Pte Ltd on SW-2026, the Sustainable Workspace Launch. HR, Marketing, Finance and Operations share one evidence trail. Launch is planned for 1 October 2026; budget SGD 18,000; target 120 qualified enquiries.
+Source: Lumina-Company-Brief.docx. Use your own reviewed prior-lab files first; scenario/ contains supplied fallback examples.
+Expectations: Save SW-2026-Source-Register.xlsx. Record source version, verified facts, unresolved questions and reviewer in Lumina-Living-Lab-01.xlsx. Keep projectSW-2026 and action IDsA01–A04 unchanged. Label every output Draft until reviewed; record actual app actions separately.</t>
   </si>
   <si>
     <t xml:space="preserve">Attached lab files only</t>
@@ -109,16 +170,10 @@
     <t xml:space="preserve">Learner</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
-  </si>
-  <si>
     <t xml:space="preserve">Evidence_ID</t>
   </si>
   <si>
     <t xml:space="preserve">Artifact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
   </si>
   <si>
     <t xml:space="preserve">Check</t>
@@ -179,7 +234,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,6 +256,20 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -303,16 +372,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -320,19 +401,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -694,144 +775,255 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="3" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="3" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="24.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="B10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H10"/>
@@ -850,7 +1042,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -858,51 +1050,51 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="3" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>26</v>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -921,7 +1113,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -929,94 +1121,94 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="3" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="3" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" s="7"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="7"/>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="10"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G5"/>
@@ -1034,7 +1226,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1042,38 +1234,38 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>